<commit_message>
markdown > s5b_ts_forecast > QMD > footnotes: Note that Quarto re-labels footnotes upon rendering, in both the rendered file and the QMD file.  I've recorded the original QMD footnote labels, since they convey the meaning of the footnote.
</commit_message>
<xml_diff>
--- a/data/xl/s5b-notes-CY25-Q2a.xlsx
+++ b/data/xl/s5b-notes-CY25-Q2a.xlsx
@@ -8,27 +8,29 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://d.docs.live.net/ca9ccbbb0bd9c947/Documents/GitHub/eda_4350/data/xl/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="360" documentId="8_{BE919223-632E-4CA3-A135-7A7680007E62}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{B7628742-AE06-4431-8B54-3F3713C8705D}"/>
+  <xr:revisionPtr revIDLastSave="467" documentId="8_{BE919223-632E-4CA3-A135-7A7680007E62}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{47E43BCA-B2FB-4B89-8666-5FC961CD5001}"/>
   <bookViews>
-    <workbookView xWindow="2100" yWindow="504" windowWidth="18858" windowHeight="11136" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="4362" yWindow="1530" windowWidth="18858" windowHeight="11136" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="index" sheetId="2" r:id="rId1"/>
-    <sheet name="eq_labels" sheetId="11" r:id="rId2"/>
-    <sheet name="templates" sheetId="1" r:id="rId3"/>
+    <sheet name="eq_labels_1" sheetId="11" r:id="rId2"/>
+    <sheet name="foot_1" sheetId="12" r:id="rId3"/>
+    <sheet name="templates" sheetId="1" r:id="rId4"/>
   </sheets>
   <externalReferences>
-    <externalReference r:id="rId4"/>
     <externalReference r:id="rId5"/>
+    <externalReference r:id="rId6"/>
   </externalReferences>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">templates!$B$5:$O$5</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="3" hidden="1">templates!$B$5:$O$5</definedName>
     <definedName name="all_Buyers">[1]pct_per_factor!$D$1:$D$65536</definedName>
     <definedName name="corr">[2]statistics!$A$2</definedName>
     <definedName name="noOct">[1]pct_per_factor!$A$6:$IV$6</definedName>
-    <definedName name="_xlnm.Print_Titles" localSheetId="1">eq_labels!$1:$1</definedName>
+    <definedName name="_xlnm.Print_Titles" localSheetId="1">eq_labels_1!$1:$1</definedName>
+    <definedName name="_xlnm.Print_Titles" localSheetId="2">foot_1!$1:$1</definedName>
     <definedName name="_xlnm.Print_Titles" localSheetId="0">index!$1:$1</definedName>
-    <definedName name="_xlnm.Print_Titles" localSheetId="2">templates!$1:$1</definedName>
+    <definedName name="_xlnm.Print_Titles" localSheetId="3">templates!$1:$1</definedName>
     <definedName name="yesOct">[1]pct_per_factor!$A$7:$IV$7</definedName>
   </definedNames>
   <calcPr calcId="191029"/>
@@ -52,7 +54,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="191" uniqueCount="149">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="226" uniqueCount="175">
   <si>
     <t>tag</t>
   </si>
@@ -498,7 +500,85 @@
     <t>revise labels of equations</t>
   </si>
   <si>
-    <t>eq_labels</t>
+    <t>eq_labels_1</t>
+  </si>
+  <si>
+    <t>foot_1</t>
+  </si>
+  <si>
+    <t>footnote labels</t>
+  </si>
+  <si>
+    <t>pg_txt</t>
+  </si>
+  <si>
+    <t>tag_foot</t>
+  </si>
+  <si>
+    <t>ts_real_valued</t>
+  </si>
+  <si>
+    <t>uni_subscripts</t>
+  </si>
+  <si>
+    <t>stationary</t>
+  </si>
+  <si>
+    <t>Gaussian</t>
+  </si>
+  <si>
+    <t>rho_even</t>
+  </si>
+  <si>
+    <t>cmort_trend_models</t>
+  </si>
+  <si>
+    <t>causal</t>
+  </si>
+  <si>
+    <t>invertible</t>
+  </si>
+  <si>
+    <t>poly_roots</t>
+  </si>
+  <si>
+    <t>MA1_transform</t>
+  </si>
+  <si>
+    <t>djia_returns</t>
+  </si>
+  <si>
+    <t>ma_simple</t>
+  </si>
+  <si>
+    <t>txt_cmort_model</t>
+  </si>
+  <si>
+    <t>txt_PACF_intro</t>
+  </si>
+  <si>
+    <t>txt_DL_algo</t>
+  </si>
+  <si>
+    <t>txt_AR1_ACF</t>
+  </si>
+  <si>
+    <t>txt_AR1_PACF</t>
+  </si>
+  <si>
+    <t>txt_causal_form</t>
+  </si>
+  <si>
+    <t>txt_MA1_equivalence</t>
+  </si>
+  <si>
+    <t>txt_MA1_ACF</t>
+  </si>
+  <si>
+    <t>idx_render</t>
+  </si>
+  <si>
+    <t>idx_src</t>
   </si>
 </sst>
 </file>
@@ -878,6 +958,10 @@
 </externalLink>
 </file>
 
+<file path=xl/persons/person.xml><?xml version="1.0" encoding="utf-8"?>
+<personList xmlns="http://schemas.microsoft.com/office/spreadsheetml/2018/threadedcomments" xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main"/>
+</file>
+
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
 <a:theme xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" name="Office Theme">
   <a:themeElements>
@@ -1141,7 +1225,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:J7"/>
+  <dimension ref="A1:J8"/>
   <sheetFormatPr defaultColWidth="9.15625" defaultRowHeight="14.4" x14ac:dyDescent="0.55000000000000004"/>
   <cols>
     <col min="1" max="1" width="1.68359375" style="1" customWidth="1"/>
@@ -1236,13 +1320,13 @@
     </row>
     <row r="7" spans="1:10" x14ac:dyDescent="0.55000000000000004">
       <c r="B7" s="1" t="s">
-        <v>45</v>
+        <v>149</v>
       </c>
       <c r="C7" s="1" t="s">
-        <v>46</v>
+        <v>150</v>
       </c>
       <c r="D7" s="30">
-        <v>45698</v>
+        <v>45827</v>
       </c>
       <c r="H7" s="1" t="s">
         <v>43</v>
@@ -1251,6 +1335,26 @@
         <v>44</v>
       </c>
       <c r="J7" s="1" t="s">
+        <v>48</v>
+      </c>
+    </row>
+    <row r="8" spans="1:10" x14ac:dyDescent="0.55000000000000004">
+      <c r="B8" s="1" t="s">
+        <v>45</v>
+      </c>
+      <c r="C8" s="1" t="s">
+        <v>46</v>
+      </c>
+      <c r="D8" s="30">
+        <v>45698</v>
+      </c>
+      <c r="H8" s="1" t="s">
+        <v>43</v>
+      </c>
+      <c r="I8" s="1" t="s">
+        <v>44</v>
+      </c>
+      <c r="J8" s="1" t="s">
         <v>48</v>
       </c>
     </row>
@@ -2296,6 +2400,294 @@
 </file>
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{1D1C1021-2470-4A18-9715-81111F931C52}">
+  <dimension ref="A1:E26"/>
+  <sheetFormatPr defaultColWidth="9.15625" defaultRowHeight="14.4" x14ac:dyDescent="0.55000000000000004"/>
+  <cols>
+    <col min="1" max="1" width="1.68359375" style="1" customWidth="1"/>
+    <col min="2" max="3" width="6.578125" style="15" customWidth="1"/>
+    <col min="4" max="4" width="21.578125" style="1" customWidth="1"/>
+    <col min="5" max="5" width="9.578125" style="15" customWidth="1"/>
+    <col min="6" max="16384" width="9.15625" style="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:5" s="2" customFormat="1" x14ac:dyDescent="0.55000000000000004">
+      <c r="A1" s="2" t="s">
+        <v>0</v>
+      </c>
+      <c r="B1" s="13" t="s">
+        <v>173</v>
+      </c>
+      <c r="C1" s="13" t="s">
+        <v>174</v>
+      </c>
+      <c r="D1" s="2" t="s">
+        <v>152</v>
+      </c>
+      <c r="E1" s="13" t="s">
+        <v>151</v>
+      </c>
+    </row>
+    <row r="2" spans="1:5" s="3" customFormat="1" ht="11.7" hidden="1" x14ac:dyDescent="0.55000000000000004">
+      <c r="A2" s="3" t="s">
+        <v>30</v>
+      </c>
+      <c r="B2" s="14"/>
+      <c r="C2" s="14"/>
+      <c r="E2" s="14"/>
+    </row>
+    <row r="3" spans="1:5" s="3" customFormat="1" ht="11.7" hidden="1" x14ac:dyDescent="0.55000000000000004">
+      <c r="A3" s="3" t="s">
+        <v>31</v>
+      </c>
+      <c r="B3" s="14"/>
+      <c r="C3" s="14"/>
+      <c r="E3" s="14"/>
+    </row>
+    <row r="4" spans="1:5" s="3" customFormat="1" ht="11.7" hidden="1" x14ac:dyDescent="0.55000000000000004">
+      <c r="A4" s="3" t="s">
+        <v>32</v>
+      </c>
+      <c r="B4" s="14"/>
+      <c r="C4" s="14"/>
+      <c r="E4" s="14"/>
+    </row>
+    <row r="5" spans="1:5" s="3" customFormat="1" ht="45" hidden="1" customHeight="1" x14ac:dyDescent="0.55000000000000004">
+      <c r="A5" s="3" t="s">
+        <v>33</v>
+      </c>
+      <c r="B5" s="14"/>
+      <c r="C5" s="14"/>
+      <c r="E5" s="14"/>
+    </row>
+    <row r="6" spans="1:5" x14ac:dyDescent="0.55000000000000004">
+      <c r="B6" s="15">
+        <v>1</v>
+      </c>
+      <c r="C6" s="15">
+        <v>1</v>
+      </c>
+      <c r="D6" s="1" t="s">
+        <v>153</v>
+      </c>
+    </row>
+    <row r="7" spans="1:5" x14ac:dyDescent="0.55000000000000004">
+      <c r="B7" s="15">
+        <v>2</v>
+      </c>
+      <c r="D7" s="1" t="s">
+        <v>154</v>
+      </c>
+    </row>
+    <row r="8" spans="1:5" x14ac:dyDescent="0.55000000000000004">
+      <c r="B8" s="15">
+        <v>3</v>
+      </c>
+      <c r="C8" s="15">
+        <v>2</v>
+      </c>
+      <c r="D8" s="1" t="s">
+        <v>155</v>
+      </c>
+    </row>
+    <row r="9" spans="1:5" x14ac:dyDescent="0.55000000000000004">
+      <c r="B9" s="15">
+        <v>4</v>
+      </c>
+      <c r="D9" s="1" t="s">
+        <v>166</v>
+      </c>
+      <c r="E9" s="15">
+        <v>108</v>
+      </c>
+    </row>
+    <row r="10" spans="1:5" x14ac:dyDescent="0.55000000000000004">
+      <c r="B10" s="15">
+        <v>5</v>
+      </c>
+      <c r="C10" s="15">
+        <v>3</v>
+      </c>
+      <c r="D10" s="1" t="s">
+        <v>156</v>
+      </c>
+    </row>
+    <row r="11" spans="1:5" x14ac:dyDescent="0.55000000000000004">
+      <c r="B11" s="15">
+        <v>6</v>
+      </c>
+      <c r="C11" s="15">
+        <v>4</v>
+      </c>
+      <c r="D11" s="1" t="s">
+        <v>157</v>
+      </c>
+    </row>
+    <row r="12" spans="1:5" x14ac:dyDescent="0.55000000000000004">
+      <c r="B12" s="15">
+        <v>7</v>
+      </c>
+      <c r="D12" s="1" t="s">
+        <v>167</v>
+      </c>
+      <c r="E12" s="15">
+        <v>115</v>
+      </c>
+    </row>
+    <row r="13" spans="1:5" x14ac:dyDescent="0.55000000000000004">
+      <c r="B13" s="15">
+        <v>8</v>
+      </c>
+      <c r="C13" s="15">
+        <v>5</v>
+      </c>
+      <c r="D13" s="1" t="s">
+        <v>164</v>
+      </c>
+    </row>
+    <row r="14" spans="1:5" x14ac:dyDescent="0.55000000000000004">
+      <c r="B14" s="15">
+        <v>9</v>
+      </c>
+      <c r="D14" s="1" t="s">
+        <v>165</v>
+      </c>
+      <c r="E14" s="15">
+        <v>55</v>
+      </c>
+    </row>
+    <row r="15" spans="1:5" x14ac:dyDescent="0.55000000000000004">
+      <c r="B15" s="15">
+        <v>10</v>
+      </c>
+      <c r="C15" s="15">
+        <v>6</v>
+      </c>
+      <c r="D15" s="1" t="s">
+        <v>158</v>
+      </c>
+    </row>
+    <row r="16" spans="1:5" x14ac:dyDescent="0.55000000000000004">
+      <c r="B16" s="15">
+        <v>11</v>
+      </c>
+      <c r="D16" s="1" t="s">
+        <v>159</v>
+      </c>
+    </row>
+    <row r="17" spans="2:5" x14ac:dyDescent="0.55000000000000004">
+      <c r="B17" s="15">
+        <v>12</v>
+      </c>
+      <c r="D17" s="1" t="s">
+        <v>160</v>
+      </c>
+    </row>
+    <row r="18" spans="2:5" x14ac:dyDescent="0.55000000000000004">
+      <c r="B18" s="15">
+        <v>13</v>
+      </c>
+      <c r="D18" s="1" t="s">
+        <v>161</v>
+      </c>
+    </row>
+    <row r="19" spans="2:5" x14ac:dyDescent="0.55000000000000004">
+      <c r="B19" s="15">
+        <v>14</v>
+      </c>
+      <c r="D19" s="1" t="s">
+        <v>168</v>
+      </c>
+      <c r="E19" s="15">
+        <v>88</v>
+      </c>
+    </row>
+    <row r="20" spans="2:5" x14ac:dyDescent="0.55000000000000004">
+      <c r="B20" s="15">
+        <v>15</v>
+      </c>
+      <c r="D20" s="1" t="s">
+        <v>169</v>
+      </c>
+      <c r="E20" s="15">
+        <v>110</v>
+      </c>
+    </row>
+    <row r="21" spans="2:5" x14ac:dyDescent="0.55000000000000004">
+      <c r="B21" s="15">
+        <v>16</v>
+      </c>
+      <c r="D21" s="1" t="s">
+        <v>170</v>
+      </c>
+      <c r="E21" s="15">
+        <v>117</v>
+      </c>
+    </row>
+    <row r="22" spans="2:5" x14ac:dyDescent="0.55000000000000004">
+      <c r="B22" s="15">
+        <v>17</v>
+      </c>
+      <c r="D22" s="1" t="s">
+        <v>171</v>
+      </c>
+      <c r="E22" s="15">
+        <v>92</v>
+      </c>
+    </row>
+    <row r="23" spans="2:5" x14ac:dyDescent="0.55000000000000004">
+      <c r="B23" s="15">
+        <v>18</v>
+      </c>
+      <c r="D23" s="1" t="s">
+        <v>162</v>
+      </c>
+    </row>
+    <row r="24" spans="2:5" x14ac:dyDescent="0.55000000000000004">
+      <c r="B24" s="15">
+        <v>19</v>
+      </c>
+      <c r="D24" s="1" t="s">
+        <v>172</v>
+      </c>
+      <c r="E24" s="15">
+        <v>93</v>
+      </c>
+    </row>
+    <row r="25" spans="2:5" x14ac:dyDescent="0.55000000000000004">
+      <c r="B25" s="15">
+        <v>20</v>
+      </c>
+      <c r="D25" s="1" t="s">
+        <v>172</v>
+      </c>
+      <c r="E25" s="15">
+        <v>111</v>
+      </c>
+    </row>
+    <row r="26" spans="2:5" x14ac:dyDescent="0.55000000000000004">
+      <c r="B26" s="15">
+        <v>21</v>
+      </c>
+      <c r="D26" s="1" t="s">
+        <v>163</v>
+      </c>
+    </row>
+  </sheetData>
+  <sortState xmlns:xlrd2="http://schemas.microsoft.com/office/spreadsheetml/2017/richdata2" ref="B6:E26">
+    <sortCondition ref="B6:B26"/>
+    <sortCondition ref="D6:D26"/>
+  </sortState>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <pageSetup orientation="landscape" r:id="rId1"/>
+  <headerFooter>
+    <oddHeader>&amp;L&amp;F&amp;CUNCLASSIFIED&amp;R&amp;A</oddHeader>
+    <oddFooter>&amp;Lprinted: &amp;D&amp;CUNCLASSIFIED&amp;Rpage &amp;P of &amp;N</oddFooter>
+  </headerFooter>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0400-000000000000}">
   <dimension ref="A1:O20"/>
   <sheetFormatPr defaultColWidth="9.15625" defaultRowHeight="14.4" x14ac:dyDescent="0.55000000000000004"/>

</xml_diff>

<commit_message>
markdown > s5b_ts_forecast > QMD > footnotes: restore origingal labels of footnotes, with the exception of the first and last footnote, labeled [^1] and [^2], respectively.  This seems to block Quarto from re-labeling the intervening footnotes.
</commit_message>
<xml_diff>
--- a/data/xl/s5b-notes-CY25-Q2a.xlsx
+++ b/data/xl/s5b-notes-CY25-Q2a.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://d.docs.live.net/ca9ccbbb0bd9c947/Documents/GitHub/eda_4350/data/xl/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="467" documentId="8_{BE919223-632E-4CA3-A135-7A7680007E62}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{47E43BCA-B2FB-4B89-8666-5FC961CD5001}"/>
+  <xr:revisionPtr revIDLastSave="469" documentId="8_{BE919223-632E-4CA3-A135-7A7680007E62}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{7BBA02B8-0C59-45F8-ADFE-A22F04204459}"/>
   <bookViews>
-    <workbookView xWindow="4362" yWindow="1530" windowWidth="18858" windowHeight="11136" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="4182" yWindow="1530" windowWidth="18858" windowHeight="11136" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="index" sheetId="2" r:id="rId1"/>
@@ -2483,9 +2483,6 @@
       <c r="B8" s="15">
         <v>3</v>
       </c>
-      <c r="C8" s="15">
-        <v>2</v>
-      </c>
       <c r="D8" s="1" t="s">
         <v>155</v>
       </c>
@@ -2505,9 +2502,6 @@
       <c r="B10" s="15">
         <v>5</v>
       </c>
-      <c r="C10" s="15">
-        <v>3</v>
-      </c>
       <c r="D10" s="1" t="s">
         <v>156</v>
       </c>
@@ -2516,9 +2510,6 @@
       <c r="B11" s="15">
         <v>6</v>
       </c>
-      <c r="C11" s="15">
-        <v>4</v>
-      </c>
       <c r="D11" s="1" t="s">
         <v>157</v>
       </c>
@@ -2538,9 +2529,6 @@
       <c r="B13" s="15">
         <v>8</v>
       </c>
-      <c r="C13" s="15">
-        <v>5</v>
-      </c>
       <c r="D13" s="1" t="s">
         <v>164</v>
       </c>
@@ -2560,9 +2548,6 @@
       <c r="B15" s="15">
         <v>10</v>
       </c>
-      <c r="C15" s="15">
-        <v>6</v>
-      </c>
       <c r="D15" s="1" t="s">
         <v>158</v>
       </c>
@@ -2668,6 +2653,9 @@
     <row r="26" spans="2:5" x14ac:dyDescent="0.55000000000000004">
       <c r="B26" s="15">
         <v>21</v>
+      </c>
+      <c r="C26" s="15">
+        <v>2</v>
       </c>
       <c r="D26" s="1" t="s">
         <v>163</v>

</xml_diff>

<commit_message>
markdown > s5b_ts_forecast > QMD > ARMA(p, q): begin section.
</commit_message>
<xml_diff>
--- a/data/xl/s5b-notes-CY25-Q2a.xlsx
+++ b/data/xl/s5b-notes-CY25-Q2a.xlsx
@@ -8,29 +8,32 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://d.docs.live.net/ca9ccbbb0bd9c947/Documents/GitHub/eda_4350/data/xl/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="469" documentId="8_{BE919223-632E-4CA3-A135-7A7680007E62}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{7BBA02B8-0C59-45F8-ADFE-A22F04204459}"/>
+  <xr:revisionPtr revIDLastSave="549" documentId="8_{BE919223-632E-4CA3-A135-7A7680007E62}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{297839CB-D59F-433C-82CA-351D90A2D111}"/>
   <bookViews>
     <workbookView xWindow="4182" yWindow="1530" windowWidth="18858" windowHeight="11136" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="index" sheetId="2" r:id="rId1"/>
     <sheet name="eq_labels_1" sheetId="11" r:id="rId2"/>
-    <sheet name="foot_1" sheetId="12" r:id="rId3"/>
-    <sheet name="templates" sheetId="1" r:id="rId4"/>
+    <sheet name="eq_labels_2" sheetId="13" r:id="rId3"/>
+    <sheet name="foot_1" sheetId="12" r:id="rId4"/>
+    <sheet name="templates" sheetId="1" r:id="rId5"/>
   </sheets>
   <externalReferences>
-    <externalReference r:id="rId5"/>
     <externalReference r:id="rId6"/>
+    <externalReference r:id="rId7"/>
   </externalReferences>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="3" hidden="1">templates!$B$5:$O$5</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="3" hidden="1">foot_1!$B$5:$E$5</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="4" hidden="1">templates!$B$5:$O$5</definedName>
     <definedName name="all_Buyers">[1]pct_per_factor!$D$1:$D$65536</definedName>
     <definedName name="corr">[2]statistics!$A$2</definedName>
     <definedName name="noOct">[1]pct_per_factor!$A$6:$IV$6</definedName>
     <definedName name="_xlnm.Print_Titles" localSheetId="1">eq_labels_1!$1:$1</definedName>
-    <definedName name="_xlnm.Print_Titles" localSheetId="2">foot_1!$1:$1</definedName>
+    <definedName name="_xlnm.Print_Titles" localSheetId="2">eq_labels_2!$1:$1</definedName>
+    <definedName name="_xlnm.Print_Titles" localSheetId="3">foot_1!$1:$1</definedName>
     <definedName name="_xlnm.Print_Titles" localSheetId="0">index!$1:$1</definedName>
-    <definedName name="_xlnm.Print_Titles" localSheetId="3">templates!$1:$1</definedName>
+    <definedName name="_xlnm.Print_Titles" localSheetId="4">templates!$1:$1</definedName>
     <definedName name="yesOct">[1]pct_per_factor!$A$7:$IV$7</definedName>
   </definedNames>
   <calcPr calcId="191029"/>
@@ -54,7 +57,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="226" uniqueCount="175">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="277" uniqueCount="179">
   <si>
     <t>tag</t>
   </si>
@@ -579,6 +582,18 @@
   </si>
   <si>
     <t>idx_src</t>
+  </si>
+  <si>
+    <t>eq_labels_2</t>
+  </si>
+  <si>
+    <t>ARMA_p_q</t>
+  </si>
+  <si>
+    <t>ARMA_1_1_not</t>
+  </si>
+  <si>
+    <t>txt_ARMA_1_1_not</t>
   </si>
 </sst>
 </file>
@@ -594,7 +609,7 @@
     <numFmt numFmtId="168" formatCode="[$-409]d\-mmm\-yyyy;@"/>
     <numFmt numFmtId="169" formatCode="h:mm;@"/>
   </numFmts>
-  <fonts count="5" x14ac:knownFonts="1">
+  <fonts count="6" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -628,6 +643,12 @@
     <font>
       <sz val="10"/>
       <color theme="1"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <sz val="8"/>
       <name val="Calibri"/>
       <family val="2"/>
       <scheme val="minor"/>
@@ -1225,7 +1246,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:J8"/>
+  <dimension ref="A1:J9"/>
   <sheetFormatPr defaultColWidth="9.15625" defaultRowHeight="14.4" x14ac:dyDescent="0.55000000000000004"/>
   <cols>
     <col min="1" max="1" width="1.68359375" style="1" customWidth="1"/>
@@ -1320,10 +1341,10 @@
     </row>
     <row r="7" spans="1:10" x14ac:dyDescent="0.55000000000000004">
       <c r="B7" s="1" t="s">
-        <v>149</v>
+        <v>175</v>
       </c>
       <c r="C7" s="1" t="s">
-        <v>150</v>
+        <v>147</v>
       </c>
       <c r="D7" s="30">
         <v>45827</v>
@@ -1340,13 +1361,13 @@
     </row>
     <row r="8" spans="1:10" x14ac:dyDescent="0.55000000000000004">
       <c r="B8" s="1" t="s">
-        <v>45</v>
+        <v>149</v>
       </c>
       <c r="C8" s="1" t="s">
-        <v>46</v>
+        <v>150</v>
       </c>
       <c r="D8" s="30">
-        <v>45698</v>
+        <v>45827</v>
       </c>
       <c r="H8" s="1" t="s">
         <v>43</v>
@@ -1358,7 +1379,28 @@
         <v>48</v>
       </c>
     </row>
+    <row r="9" spans="1:10" x14ac:dyDescent="0.55000000000000004">
+      <c r="B9" s="1" t="s">
+        <v>45</v>
+      </c>
+      <c r="C9" s="1" t="s">
+        <v>46</v>
+      </c>
+      <c r="D9" s="30">
+        <v>45698</v>
+      </c>
+      <c r="H9" s="1" t="s">
+        <v>43</v>
+      </c>
+      <c r="I9" s="1" t="s">
+        <v>44</v>
+      </c>
+      <c r="J9" s="1" t="s">
+        <v>48</v>
+      </c>
+    </row>
   </sheetData>
+  <phoneticPr fontId="5" type="noConversion"/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup orientation="landscape" r:id="rId1"/>
   <headerFooter>
@@ -2400,8 +2442,368 @@
 </file>
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{19852245-2EA1-45B6-8988-FC67FD9B6DC5}">
+  <dimension ref="A1:C43"/>
+  <sheetFormatPr defaultColWidth="9.15625" defaultRowHeight="14.4" x14ac:dyDescent="0.55000000000000004"/>
+  <cols>
+    <col min="1" max="1" width="1.68359375" style="1" customWidth="1"/>
+    <col min="2" max="2" width="6.578125" style="15" customWidth="1"/>
+    <col min="3" max="3" width="21.578125" style="1" customWidth="1"/>
+    <col min="4" max="16384" width="9.15625" style="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:3" s="2" customFormat="1" x14ac:dyDescent="0.55000000000000004">
+      <c r="A1" s="2" t="s">
+        <v>0</v>
+      </c>
+      <c r="B1" s="13" t="s">
+        <v>173</v>
+      </c>
+      <c r="C1" s="2" t="s">
+        <v>96</v>
+      </c>
+    </row>
+    <row r="2" spans="1:3" s="3" customFormat="1" ht="11.7" hidden="1" x14ac:dyDescent="0.55000000000000004">
+      <c r="A2" s="3" t="s">
+        <v>30</v>
+      </c>
+      <c r="B2" s="14"/>
+    </row>
+    <row r="3" spans="1:3" s="3" customFormat="1" ht="11.7" hidden="1" x14ac:dyDescent="0.55000000000000004">
+      <c r="A3" s="3" t="s">
+        <v>31</v>
+      </c>
+      <c r="B3" s="14"/>
+    </row>
+    <row r="4" spans="1:3" s="3" customFormat="1" ht="11.7" hidden="1" x14ac:dyDescent="0.55000000000000004">
+      <c r="A4" s="3" t="s">
+        <v>32</v>
+      </c>
+      <c r="B4" s="14"/>
+    </row>
+    <row r="5" spans="1:3" s="3" customFormat="1" ht="45" hidden="1" customHeight="1" x14ac:dyDescent="0.55000000000000004">
+      <c r="A5" s="3" t="s">
+        <v>33</v>
+      </c>
+      <c r="B5" s="14"/>
+    </row>
+    <row r="6" spans="1:3" x14ac:dyDescent="0.55000000000000004">
+      <c r="B6" s="15">
+        <v>1</v>
+      </c>
+      <c r="C6" s="1" t="s">
+        <v>117</v>
+      </c>
+    </row>
+    <row r="7" spans="1:3" x14ac:dyDescent="0.55000000000000004">
+      <c r="B7" s="15">
+        <v>2</v>
+      </c>
+      <c r="C7" s="1" t="s">
+        <v>118</v>
+      </c>
+    </row>
+    <row r="8" spans="1:3" x14ac:dyDescent="0.55000000000000004">
+      <c r="B8" s="15">
+        <v>3</v>
+      </c>
+      <c r="C8" s="1" t="s">
+        <v>99</v>
+      </c>
+    </row>
+    <row r="9" spans="1:3" x14ac:dyDescent="0.55000000000000004">
+      <c r="B9" s="15">
+        <v>4</v>
+      </c>
+      <c r="C9" s="1" t="s">
+        <v>119</v>
+      </c>
+    </row>
+    <row r="10" spans="1:3" x14ac:dyDescent="0.55000000000000004">
+      <c r="B10" s="15">
+        <v>5</v>
+      </c>
+      <c r="C10" s="1" t="s">
+        <v>100</v>
+      </c>
+    </row>
+    <row r="11" spans="1:3" x14ac:dyDescent="0.55000000000000004">
+      <c r="B11" s="15">
+        <v>6</v>
+      </c>
+      <c r="C11" s="1" t="s">
+        <v>101</v>
+      </c>
+    </row>
+    <row r="12" spans="1:3" x14ac:dyDescent="0.55000000000000004">
+      <c r="B12" s="15">
+        <v>7</v>
+      </c>
+      <c r="C12" s="1" t="s">
+        <v>102</v>
+      </c>
+    </row>
+    <row r="13" spans="1:3" x14ac:dyDescent="0.55000000000000004">
+      <c r="B13" s="15">
+        <v>8</v>
+      </c>
+      <c r="C13" s="1" t="s">
+        <v>103</v>
+      </c>
+    </row>
+    <row r="14" spans="1:3" x14ac:dyDescent="0.55000000000000004">
+      <c r="B14" s="15">
+        <v>9</v>
+      </c>
+      <c r="C14" s="1" t="s">
+        <v>104</v>
+      </c>
+    </row>
+    <row r="15" spans="1:3" x14ac:dyDescent="0.55000000000000004">
+      <c r="B15" s="15">
+        <v>10</v>
+      </c>
+      <c r="C15" s="1" t="s">
+        <v>120</v>
+      </c>
+    </row>
+    <row r="16" spans="1:3" x14ac:dyDescent="0.55000000000000004">
+      <c r="B16" s="15">
+        <v>11</v>
+      </c>
+      <c r="C16" s="1" t="s">
+        <v>121</v>
+      </c>
+    </row>
+    <row r="17" spans="2:3" x14ac:dyDescent="0.55000000000000004">
+      <c r="B17" s="15">
+        <v>12</v>
+      </c>
+      <c r="C17" s="1" t="s">
+        <v>105</v>
+      </c>
+    </row>
+    <row r="18" spans="2:3" x14ac:dyDescent="0.55000000000000004">
+      <c r="B18" s="15">
+        <v>13</v>
+      </c>
+      <c r="C18" s="1" t="s">
+        <v>122</v>
+      </c>
+    </row>
+    <row r="19" spans="2:3" x14ac:dyDescent="0.55000000000000004">
+      <c r="B19" s="15">
+        <v>14</v>
+      </c>
+      <c r="C19" s="1" t="s">
+        <v>123</v>
+      </c>
+    </row>
+    <row r="20" spans="2:3" x14ac:dyDescent="0.55000000000000004">
+      <c r="B20" s="15">
+        <v>15</v>
+      </c>
+      <c r="C20" s="1" t="s">
+        <v>124</v>
+      </c>
+    </row>
+    <row r="21" spans="2:3" x14ac:dyDescent="0.55000000000000004">
+      <c r="B21" s="15">
+        <v>16</v>
+      </c>
+      <c r="C21" s="1" t="s">
+        <v>125</v>
+      </c>
+    </row>
+    <row r="22" spans="2:3" x14ac:dyDescent="0.55000000000000004">
+      <c r="B22" s="15">
+        <v>17</v>
+      </c>
+      <c r="C22" s="1" t="s">
+        <v>106</v>
+      </c>
+    </row>
+    <row r="23" spans="2:3" x14ac:dyDescent="0.55000000000000004">
+      <c r="B23" s="15">
+        <v>18</v>
+      </c>
+      <c r="C23" s="1" t="s">
+        <v>126</v>
+      </c>
+    </row>
+    <row r="24" spans="2:3" x14ac:dyDescent="0.55000000000000004">
+      <c r="B24" s="15">
+        <v>19</v>
+      </c>
+      <c r="C24" s="1" t="s">
+        <v>107</v>
+      </c>
+    </row>
+    <row r="25" spans="2:3" x14ac:dyDescent="0.55000000000000004">
+      <c r="B25" s="15">
+        <v>20</v>
+      </c>
+      <c r="C25" s="1" t="s">
+        <v>108</v>
+      </c>
+    </row>
+    <row r="26" spans="2:3" x14ac:dyDescent="0.55000000000000004">
+      <c r="B26" s="15">
+        <v>21</v>
+      </c>
+      <c r="C26" s="1" t="s">
+        <v>127</v>
+      </c>
+    </row>
+    <row r="27" spans="2:3" x14ac:dyDescent="0.55000000000000004">
+      <c r="B27" s="15">
+        <v>22</v>
+      </c>
+      <c r="C27" s="1" t="s">
+        <v>109</v>
+      </c>
+    </row>
+    <row r="28" spans="2:3" x14ac:dyDescent="0.55000000000000004">
+      <c r="B28" s="15">
+        <v>23</v>
+      </c>
+      <c r="C28" s="1" t="s">
+        <v>128</v>
+      </c>
+    </row>
+    <row r="29" spans="2:3" x14ac:dyDescent="0.55000000000000004">
+      <c r="B29" s="15">
+        <v>24</v>
+      </c>
+      <c r="C29" s="1" t="s">
+        <v>129</v>
+      </c>
+    </row>
+    <row r="30" spans="2:3" x14ac:dyDescent="0.55000000000000004">
+      <c r="B30" s="15">
+        <v>25</v>
+      </c>
+      <c r="C30" s="1" t="s">
+        <v>110</v>
+      </c>
+    </row>
+    <row r="31" spans="2:3" x14ac:dyDescent="0.55000000000000004">
+      <c r="B31" s="15">
+        <v>26</v>
+      </c>
+      <c r="C31" s="1" t="s">
+        <v>112</v>
+      </c>
+    </row>
+    <row r="32" spans="2:3" x14ac:dyDescent="0.55000000000000004">
+      <c r="B32" s="15">
+        <v>27</v>
+      </c>
+      <c r="C32" s="1" t="s">
+        <v>111</v>
+      </c>
+    </row>
+    <row r="33" spans="2:3" x14ac:dyDescent="0.55000000000000004">
+      <c r="B33" s="15">
+        <v>28</v>
+      </c>
+      <c r="C33" s="1" t="s">
+        <v>130</v>
+      </c>
+    </row>
+    <row r="34" spans="2:3" x14ac:dyDescent="0.55000000000000004">
+      <c r="B34" s="15">
+        <v>29</v>
+      </c>
+      <c r="C34" s="1" t="s">
+        <v>131</v>
+      </c>
+    </row>
+    <row r="35" spans="2:3" x14ac:dyDescent="0.55000000000000004">
+      <c r="B35" s="15">
+        <v>30</v>
+      </c>
+      <c r="C35" s="1" t="s">
+        <v>132</v>
+      </c>
+    </row>
+    <row r="36" spans="2:3" x14ac:dyDescent="0.55000000000000004">
+      <c r="B36" s="15">
+        <v>31</v>
+      </c>
+      <c r="C36" s="1" t="s">
+        <v>133</v>
+      </c>
+    </row>
+    <row r="37" spans="2:3" x14ac:dyDescent="0.55000000000000004">
+      <c r="B37" s="15">
+        <v>32</v>
+      </c>
+      <c r="C37" s="1" t="s">
+        <v>113</v>
+      </c>
+    </row>
+    <row r="38" spans="2:3" x14ac:dyDescent="0.55000000000000004">
+      <c r="B38" s="15">
+        <v>33</v>
+      </c>
+      <c r="C38" s="1" t="s">
+        <v>114</v>
+      </c>
+    </row>
+    <row r="39" spans="2:3" x14ac:dyDescent="0.55000000000000004">
+      <c r="B39" s="15">
+        <v>34</v>
+      </c>
+      <c r="C39" s="1" t="s">
+        <v>134</v>
+      </c>
+    </row>
+    <row r="40" spans="2:3" x14ac:dyDescent="0.55000000000000004">
+      <c r="B40" s="15">
+        <v>35</v>
+      </c>
+      <c r="C40" s="1" t="s">
+        <v>135</v>
+      </c>
+    </row>
+    <row r="41" spans="2:3" x14ac:dyDescent="0.55000000000000004">
+      <c r="B41" s="15">
+        <v>36</v>
+      </c>
+      <c r="C41" s="1" t="s">
+        <v>136</v>
+      </c>
+    </row>
+    <row r="42" spans="2:3" x14ac:dyDescent="0.55000000000000004">
+      <c r="B42" s="15">
+        <v>37</v>
+      </c>
+      <c r="C42" s="1" t="s">
+        <v>176</v>
+      </c>
+    </row>
+    <row r="43" spans="2:3" x14ac:dyDescent="0.55000000000000004">
+      <c r="B43" s="15">
+        <v>38</v>
+      </c>
+      <c r="C43" s="1" t="s">
+        <v>177</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <pageSetup orientation="landscape" r:id="rId1"/>
+  <headerFooter>
+    <oddHeader>&amp;L&amp;F&amp;CUNCLASSIFIED&amp;R&amp;A</oddHeader>
+    <oddFooter>&amp;Lprinted: &amp;D&amp;CUNCLASSIFIED&amp;Rpage &amp;P of &amp;N</oddFooter>
+  </headerFooter>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{1D1C1021-2470-4A18-9715-81111F931C52}">
-  <dimension ref="A1:E26"/>
+  <dimension ref="A1:E27"/>
   <sheetFormatPr defaultColWidth="9.15625" defaultRowHeight="14.4" x14ac:dyDescent="0.55000000000000004"/>
   <cols>
     <col min="1" max="1" width="1.68359375" style="1" customWidth="1"/>
@@ -2452,7 +2854,7 @@
       <c r="C4" s="14"/>
       <c r="E4" s="14"/>
     </row>
-    <row r="5" spans="1:5" s="3" customFormat="1" ht="45" hidden="1" customHeight="1" x14ac:dyDescent="0.55000000000000004">
+    <row r="5" spans="1:5" s="3" customFormat="1" ht="45" customHeight="1" x14ac:dyDescent="0.55000000000000004">
       <c r="A5" s="3" t="s">
         <v>33</v>
       </c>
@@ -2654,17 +3056,30 @@
       <c r="B26" s="15">
         <v>21</v>
       </c>
-      <c r="C26" s="15">
+      <c r="D26" s="1" t="s">
+        <v>178</v>
+      </c>
+      <c r="E26" s="15">
+        <v>95</v>
+      </c>
+    </row>
+    <row r="27" spans="2:5" x14ac:dyDescent="0.55000000000000004">
+      <c r="B27" s="15">
+        <v>22</v>
+      </c>
+      <c r="C27" s="15">
         <v>2</v>
       </c>
-      <c r="D26" s="1" t="s">
+      <c r="D27" s="1" t="s">
         <v>163</v>
       </c>
     </row>
   </sheetData>
-  <sortState xmlns:xlrd2="http://schemas.microsoft.com/office/spreadsheetml/2017/richdata2" ref="B6:E26">
-    <sortCondition ref="B6:B26"/>
-    <sortCondition ref="D6:D26"/>
+  <autoFilter ref="B5:E5" xr:uid="{1D1C1021-2470-4A18-9715-81111F931C52}"/>
+  <sortState xmlns:xlrd2="http://schemas.microsoft.com/office/spreadsheetml/2017/richdata2" ref="B6:E27">
+    <sortCondition ref="B6:B27"/>
+    <sortCondition ref="D6:D27"/>
+    <sortCondition ref="E6:E27"/>
   </sortState>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup orientation="landscape" r:id="rId1"/>
@@ -2675,7 +3090,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0400-000000000000}">
   <dimension ref="A1:O20"/>
   <sheetFormatPr defaultColWidth="9.15625" defaultRowHeight="14.4" x14ac:dyDescent="0.55000000000000004"/>

</xml_diff>

<commit_message>
markdown > s5b_ts_forecast.QMD: restore footnotes that were overwritten by the editor in the cursed Visual mode (herewith banned by the YAML command "editor: source").
</commit_message>
<xml_diff>
--- a/data/xl/s5b-notes-CY25-Q2a.xlsx
+++ b/data/xl/s5b-notes-CY25-Q2a.xlsx
@@ -1,39 +1,42 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="28827"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="28925"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://d.docs.live.net/ca9ccbbb0bd9c947/Documents/GitHub/eda_4350/data/xl/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="549" documentId="8_{BE919223-632E-4CA3-A135-7A7680007E62}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{297839CB-D59F-433C-82CA-351D90A2D111}"/>
+  <xr:revisionPtr revIDLastSave="627" documentId="8_{BE919223-632E-4CA3-A135-7A7680007E62}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{0C43D3C0-B632-48D7-9AEA-C7A883C071C6}"/>
   <bookViews>
-    <workbookView xWindow="4182" yWindow="1530" windowWidth="18858" windowHeight="11136" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="786" yWindow="138" windowWidth="18858" windowHeight="11136" activeTab="4" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="index" sheetId="2" r:id="rId1"/>
     <sheet name="eq_labels_1" sheetId="11" r:id="rId2"/>
     <sheet name="eq_labels_2" sheetId="13" r:id="rId3"/>
     <sheet name="foot_1" sheetId="12" r:id="rId4"/>
-    <sheet name="templates" sheetId="1" r:id="rId5"/>
+    <sheet name="foot_2" sheetId="14" r:id="rId5"/>
+    <sheet name="templates" sheetId="1" r:id="rId6"/>
   </sheets>
   <externalReferences>
-    <externalReference r:id="rId6"/>
     <externalReference r:id="rId7"/>
+    <externalReference r:id="rId8"/>
   </externalReferences>
   <definedNames>
     <definedName name="_xlnm._FilterDatabase" localSheetId="3" hidden="1">foot_1!$B$5:$E$5</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="4" hidden="1">templates!$B$5:$O$5</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="4" hidden="1">foot_2!$B$5:$E$5</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="5" hidden="1">templates!$B$5:$O$5</definedName>
     <definedName name="all_Buyers">[1]pct_per_factor!$D$1:$D$65536</definedName>
     <definedName name="corr">[2]statistics!$A$2</definedName>
     <definedName name="noOct">[1]pct_per_factor!$A$6:$IV$6</definedName>
     <definedName name="_xlnm.Print_Titles" localSheetId="1">eq_labels_1!$1:$1</definedName>
     <definedName name="_xlnm.Print_Titles" localSheetId="2">eq_labels_2!$1:$1</definedName>
     <definedName name="_xlnm.Print_Titles" localSheetId="3">foot_1!$1:$1</definedName>
+    <definedName name="_xlnm.Print_Titles" localSheetId="4">foot_2!$1:$1</definedName>
     <definedName name="_xlnm.Print_Titles" localSheetId="0">index!$1:$1</definedName>
-    <definedName name="_xlnm.Print_Titles" localSheetId="4">templates!$1:$1</definedName>
+    <definedName name="_xlnm.Print_Titles" localSheetId="5">templates!$1:$1</definedName>
     <definedName name="yesOct">[1]pct_per_factor!$A$7:$IV$7</definedName>
   </definedNames>
   <calcPr calcId="191029"/>
@@ -57,7 +60,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="277" uniqueCount="179">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="345" uniqueCount="230">
   <si>
     <t>tag</t>
   </si>
@@ -594,6 +597,159 @@
   </si>
   <si>
     <t>txt_ARMA_1_1_not</t>
+  </si>
+  <si>
+    <t>non-Gaussian</t>
+  </si>
+  <si>
+    <t>ts-real-valued</t>
+  </si>
+  <si>
+    <t>uni-subscripts</t>
+  </si>
+  <si>
+    <t>txt-PACF-intro</t>
+  </si>
+  <si>
+    <t>rho-even</t>
+  </si>
+  <si>
+    <t>txt-DL-algo</t>
+  </si>
+  <si>
+    <t>txt-cmort-model</t>
+  </si>
+  <si>
+    <t>cmort-trend-models</t>
+  </si>
+  <si>
+    <t>poly-roots</t>
+  </si>
+  <si>
+    <t>txt-AR1-ACF</t>
+  </si>
+  <si>
+    <t>txt-AR1-PACF</t>
+  </si>
+  <si>
+    <t>txt-MA1-ACF</t>
+  </si>
+  <si>
+    <t>djia-returns</t>
+  </si>
+  <si>
+    <t>txt-PACF-defn</t>
+  </si>
+  <si>
+    <t>txt-seasonal-diff</t>
+  </si>
+  <si>
+    <t>caveat-filter</t>
+  </si>
+  <si>
+    <t>txt-ARp-inverse</t>
+  </si>
+  <si>
+    <t>txt-MA1-roots</t>
+  </si>
+  <si>
+    <t>MA1-roots</t>
+  </si>
+  <si>
+    <t>txt-MA1-rho</t>
+  </si>
+  <si>
+    <t>txt-co-prime-polys</t>
+  </si>
+  <si>
+    <t>txt-ARMApq-causal</t>
+  </si>
+  <si>
+    <t>ARMApq-causal</t>
+  </si>
+  <si>
+    <t>txt-ARMApq-inverted-form</t>
+  </si>
+  <si>
+    <t>ARMApq-inverted-form</t>
+  </si>
+  <si>
+    <t>txt-Gamma-matrix</t>
+  </si>
+  <si>
+    <t>singular-Gamma-matrix</t>
+  </si>
+  <si>
+    <t>ACF-est-limitations</t>
+  </si>
+  <si>
+    <t>txt-ARMA-forecasting</t>
+  </si>
+  <si>
+    <t>e-future-given-past-notation</t>
+  </si>
+  <si>
+    <t>mspe-caveat</t>
+  </si>
+  <si>
+    <t>txt-trunc-predict</t>
+  </si>
+  <si>
+    <t>txt-ARMA_1_1_sim</t>
+  </si>
+  <si>
+    <t>txt-var-predictor-resid</t>
+  </si>
+  <si>
+    <t>var-predictor-resid</t>
+  </si>
+  <si>
+    <t>sarima-sim-script</t>
+  </si>
+  <si>
+    <t>txt-ARIMApdq</t>
+  </si>
+  <si>
+    <t>diff-is-AR1</t>
+  </si>
+  <si>
+    <t>txt-ARIMA-0-1-1</t>
+  </si>
+  <si>
+    <t>txt-SES-as-projection</t>
+  </si>
+  <si>
+    <t>sec. B.1</t>
+  </si>
+  <si>
+    <t>comment</t>
+  </si>
+  <si>
+    <t>empty-sum</t>
+  </si>
+  <si>
+    <t>book-ETS</t>
+  </si>
+  <si>
+    <t>art-Holt-Winters</t>
+  </si>
+  <si>
+    <t>ETS-ANN-ss-wn</t>
+  </si>
+  <si>
+    <t>book-ETS-category</t>
+  </si>
+  <si>
+    <t>txt-SARIMA-models</t>
+  </si>
+  <si>
+    <t>txt-cardox-xmpl</t>
+  </si>
+  <si>
+    <t>book-DRB-TSDAT</t>
+  </si>
+  <si>
+    <t>foot_2</t>
   </si>
 </sst>
 </file>
@@ -1246,7 +1402,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:J9"/>
+  <dimension ref="A1:J10"/>
   <sheetFormatPr defaultColWidth="9.15625" defaultRowHeight="14.4" x14ac:dyDescent="0.55000000000000004"/>
   <cols>
     <col min="1" max="1" width="1.68359375" style="1" customWidth="1"/>
@@ -1381,13 +1537,13 @@
     </row>
     <row r="9" spans="1:10" x14ac:dyDescent="0.55000000000000004">
       <c r="B9" s="1" t="s">
-        <v>45</v>
+        <v>229</v>
       </c>
       <c r="C9" s="1" t="s">
-        <v>46</v>
+        <v>150</v>
       </c>
       <c r="D9" s="30">
-        <v>45698</v>
+        <v>45845</v>
       </c>
       <c r="H9" s="1" t="s">
         <v>43</v>
@@ -1396,6 +1552,26 @@
         <v>44</v>
       </c>
       <c r="J9" s="1" t="s">
+        <v>48</v>
+      </c>
+    </row>
+    <row r="10" spans="1:10" x14ac:dyDescent="0.55000000000000004">
+      <c r="B10" s="1" t="s">
+        <v>45</v>
+      </c>
+      <c r="C10" s="1" t="s">
+        <v>46</v>
+      </c>
+      <c r="D10" s="30">
+        <v>45698</v>
+      </c>
+      <c r="H10" s="1" t="s">
+        <v>43</v>
+      </c>
+      <c r="I10" s="1" t="s">
+        <v>44</v>
+      </c>
+      <c r="J10" s="1" t="s">
         <v>48</v>
       </c>
     </row>
@@ -3091,6 +3267,578 @@
 </file>
 
 <file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{BF8ACCCA-78CA-47A0-A1F3-6B11447BE5E1}">
+  <dimension ref="A1:F57"/>
+  <sheetFormatPr defaultColWidth="9.15625" defaultRowHeight="14.4" x14ac:dyDescent="0.55000000000000004"/>
+  <cols>
+    <col min="1" max="1" width="1.68359375" style="1" customWidth="1"/>
+    <col min="2" max="3" width="6.578125" style="15" customWidth="1"/>
+    <col min="4" max="4" width="21.578125" style="1" customWidth="1"/>
+    <col min="5" max="5" width="9.578125" style="15" customWidth="1"/>
+    <col min="6" max="16384" width="9.15625" style="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:6" s="2" customFormat="1" x14ac:dyDescent="0.55000000000000004">
+      <c r="A1" s="2" t="s">
+        <v>0</v>
+      </c>
+      <c r="B1" s="13" t="s">
+        <v>173</v>
+      </c>
+      <c r="C1" s="13" t="s">
+        <v>174</v>
+      </c>
+      <c r="D1" s="2" t="s">
+        <v>152</v>
+      </c>
+      <c r="E1" s="13" t="s">
+        <v>151</v>
+      </c>
+      <c r="F1" s="2" t="s">
+        <v>220</v>
+      </c>
+    </row>
+    <row r="2" spans="1:6" s="3" customFormat="1" ht="11.7" hidden="1" x14ac:dyDescent="0.55000000000000004">
+      <c r="A2" s="3" t="s">
+        <v>30</v>
+      </c>
+      <c r="B2" s="14"/>
+      <c r="C2" s="14"/>
+      <c r="E2" s="14"/>
+    </row>
+    <row r="3" spans="1:6" s="3" customFormat="1" ht="11.7" hidden="1" x14ac:dyDescent="0.55000000000000004">
+      <c r="A3" s="3" t="s">
+        <v>31</v>
+      </c>
+      <c r="B3" s="14"/>
+      <c r="C3" s="14"/>
+      <c r="E3" s="14"/>
+    </row>
+    <row r="4" spans="1:6" s="3" customFormat="1" ht="11.7" hidden="1" x14ac:dyDescent="0.55000000000000004">
+      <c r="A4" s="3" t="s">
+        <v>32</v>
+      </c>
+      <c r="B4" s="14"/>
+      <c r="C4" s="14"/>
+      <c r="E4" s="14"/>
+    </row>
+    <row r="5" spans="1:6" s="3" customFormat="1" ht="45" customHeight="1" x14ac:dyDescent="0.55000000000000004">
+      <c r="A5" s="3" t="s">
+        <v>33</v>
+      </c>
+      <c r="B5" s="14"/>
+      <c r="C5" s="14"/>
+      <c r="E5" s="14"/>
+    </row>
+    <row r="6" spans="1:6" x14ac:dyDescent="0.55000000000000004">
+      <c r="B6" s="15">
+        <v>1</v>
+      </c>
+      <c r="C6" s="15">
+        <v>1001</v>
+      </c>
+      <c r="D6" s="1" t="s">
+        <v>180</v>
+      </c>
+    </row>
+    <row r="7" spans="1:6" x14ac:dyDescent="0.55000000000000004">
+      <c r="B7" s="15">
+        <v>2</v>
+      </c>
+      <c r="D7" s="1" t="s">
+        <v>181</v>
+      </c>
+    </row>
+    <row r="8" spans="1:6" x14ac:dyDescent="0.55000000000000004">
+      <c r="B8" s="15">
+        <v>3</v>
+      </c>
+      <c r="D8" s="1" t="s">
+        <v>155</v>
+      </c>
+    </row>
+    <row r="9" spans="1:6" x14ac:dyDescent="0.55000000000000004">
+      <c r="B9" s="15">
+        <v>4</v>
+      </c>
+      <c r="D9" s="1" t="s">
+        <v>182</v>
+      </c>
+      <c r="E9" s="15">
+        <v>108</v>
+      </c>
+    </row>
+    <row r="10" spans="1:6" x14ac:dyDescent="0.55000000000000004">
+      <c r="B10" s="15">
+        <v>5</v>
+      </c>
+      <c r="D10" s="1" t="s">
+        <v>156</v>
+      </c>
+    </row>
+    <row r="11" spans="1:6" x14ac:dyDescent="0.55000000000000004">
+      <c r="B11" s="15">
+        <v>6</v>
+      </c>
+      <c r="D11" s="1" t="s">
+        <v>179</v>
+      </c>
+    </row>
+    <row r="12" spans="1:6" x14ac:dyDescent="0.55000000000000004">
+      <c r="B12" s="15">
+        <v>7</v>
+      </c>
+      <c r="D12" s="1" t="s">
+        <v>183</v>
+      </c>
+    </row>
+    <row r="13" spans="1:6" x14ac:dyDescent="0.55000000000000004">
+      <c r="B13" s="15">
+        <v>8</v>
+      </c>
+      <c r="D13" s="1" t="s">
+        <v>192</v>
+      </c>
+      <c r="E13" s="15">
+        <v>110</v>
+      </c>
+    </row>
+    <row r="14" spans="1:6" x14ac:dyDescent="0.55000000000000004">
+      <c r="B14" s="15">
+        <v>9</v>
+      </c>
+      <c r="D14" s="1" t="s">
+        <v>184</v>
+      </c>
+      <c r="E14" s="15">
+        <v>115</v>
+      </c>
+    </row>
+    <row r="15" spans="1:6" x14ac:dyDescent="0.55000000000000004">
+      <c r="B15" s="15">
+        <v>10</v>
+      </c>
+      <c r="D15" s="1" t="s">
+        <v>193</v>
+      </c>
+      <c r="E15" s="15">
+        <v>157</v>
+      </c>
+    </row>
+    <row r="16" spans="1:6" x14ac:dyDescent="0.55000000000000004">
+      <c r="B16" s="15">
+        <v>11</v>
+      </c>
+      <c r="D16" s="1" t="s">
+        <v>194</v>
+      </c>
+    </row>
+    <row r="17" spans="2:5" x14ac:dyDescent="0.55000000000000004">
+      <c r="B17" s="15">
+        <v>12</v>
+      </c>
+      <c r="D17" s="1" t="s">
+        <v>185</v>
+      </c>
+      <c r="E17" s="15">
+        <v>55</v>
+      </c>
+    </row>
+    <row r="18" spans="2:5" x14ac:dyDescent="0.55000000000000004">
+      <c r="B18" s="15">
+        <v>13</v>
+      </c>
+      <c r="D18" s="1" t="s">
+        <v>186</v>
+      </c>
+    </row>
+    <row r="19" spans="2:5" x14ac:dyDescent="0.55000000000000004">
+      <c r="B19" s="15">
+        <v>14</v>
+      </c>
+      <c r="D19" s="1" t="s">
+        <v>159</v>
+      </c>
+    </row>
+    <row r="20" spans="2:5" x14ac:dyDescent="0.55000000000000004">
+      <c r="B20" s="15">
+        <v>15</v>
+      </c>
+      <c r="D20" s="1" t="s">
+        <v>160</v>
+      </c>
+    </row>
+    <row r="21" spans="2:5" x14ac:dyDescent="0.55000000000000004">
+      <c r="B21" s="15">
+        <v>16</v>
+      </c>
+      <c r="D21" s="1" t="s">
+        <v>187</v>
+      </c>
+    </row>
+    <row r="22" spans="2:5" x14ac:dyDescent="0.55000000000000004">
+      <c r="B22" s="15">
+        <v>17</v>
+      </c>
+      <c r="D22" s="1" t="s">
+        <v>188</v>
+      </c>
+      <c r="E22" s="15">
+        <v>88</v>
+      </c>
+    </row>
+    <row r="23" spans="2:5" x14ac:dyDescent="0.55000000000000004">
+      <c r="B23" s="15">
+        <v>18</v>
+      </c>
+      <c r="D23" s="1" t="s">
+        <v>189</v>
+      </c>
+      <c r="E23" s="15">
+        <v>110</v>
+      </c>
+    </row>
+    <row r="24" spans="2:5" x14ac:dyDescent="0.55000000000000004">
+      <c r="B24" s="15">
+        <v>19</v>
+      </c>
+      <c r="D24" s="1" t="s">
+        <v>195</v>
+      </c>
+      <c r="E24" s="15">
+        <v>117</v>
+      </c>
+    </row>
+    <row r="25" spans="2:5" x14ac:dyDescent="0.55000000000000004">
+      <c r="B25" s="15">
+        <v>20</v>
+      </c>
+      <c r="D25" s="1" t="s">
+        <v>196</v>
+      </c>
+      <c r="E25" s="15">
+        <v>92</v>
+      </c>
+    </row>
+    <row r="26" spans="2:5" x14ac:dyDescent="0.55000000000000004">
+      <c r="B26" s="15">
+        <v>21</v>
+      </c>
+      <c r="D26" s="1" t="s">
+        <v>197</v>
+      </c>
+    </row>
+    <row r="27" spans="2:5" x14ac:dyDescent="0.55000000000000004">
+      <c r="B27" s="15">
+        <v>22</v>
+      </c>
+      <c r="D27" s="1" t="s">
+        <v>190</v>
+      </c>
+      <c r="E27" s="15">
+        <v>93</v>
+      </c>
+    </row>
+    <row r="28" spans="2:5" x14ac:dyDescent="0.55000000000000004">
+      <c r="B28" s="15">
+        <v>23</v>
+      </c>
+      <c r="D28" s="1" t="s">
+        <v>198</v>
+      </c>
+      <c r="E28" s="15">
+        <v>111</v>
+      </c>
+    </row>
+    <row r="29" spans="2:5" x14ac:dyDescent="0.55000000000000004">
+      <c r="B29" s="15">
+        <v>24</v>
+      </c>
+      <c r="D29" s="1" t="s">
+        <v>199</v>
+      </c>
+      <c r="E29" s="15">
+        <v>95</v>
+      </c>
+    </row>
+    <row r="30" spans="2:5" x14ac:dyDescent="0.55000000000000004">
+      <c r="B30" s="15">
+        <v>25</v>
+      </c>
+      <c r="D30" s="1" t="s">
+        <v>200</v>
+      </c>
+      <c r="E30" s="15">
+        <v>97</v>
+      </c>
+    </row>
+    <row r="31" spans="2:5" x14ac:dyDescent="0.55000000000000004">
+      <c r="B31" s="15">
+        <v>26</v>
+      </c>
+      <c r="D31" s="1" t="s">
+        <v>201</v>
+      </c>
+    </row>
+    <row r="32" spans="2:5" x14ac:dyDescent="0.55000000000000004">
+      <c r="B32" s="15">
+        <v>27</v>
+      </c>
+      <c r="D32" s="1" t="s">
+        <v>202</v>
+      </c>
+      <c r="E32" s="15">
+        <v>97</v>
+      </c>
+    </row>
+    <row r="33" spans="2:6" x14ac:dyDescent="0.55000000000000004">
+      <c r="B33" s="15">
+        <v>28</v>
+      </c>
+      <c r="D33" s="1" t="s">
+        <v>203</v>
+      </c>
+    </row>
+    <row r="34" spans="2:6" x14ac:dyDescent="0.55000000000000004">
+      <c r="B34" s="15">
+        <v>29</v>
+      </c>
+      <c r="D34" s="1" t="s">
+        <v>204</v>
+      </c>
+      <c r="E34" s="15">
+        <v>114</v>
+      </c>
+    </row>
+    <row r="35" spans="2:6" x14ac:dyDescent="0.55000000000000004">
+      <c r="B35" s="15">
+        <v>30</v>
+      </c>
+      <c r="D35" s="1" t="s">
+        <v>205</v>
+      </c>
+    </row>
+    <row r="36" spans="2:6" x14ac:dyDescent="0.55000000000000004">
+      <c r="B36" s="15">
+        <v>31</v>
+      </c>
+      <c r="D36" s="1" t="s">
+        <v>206</v>
+      </c>
+    </row>
+    <row r="37" spans="2:6" x14ac:dyDescent="0.55000000000000004">
+      <c r="B37" s="15">
+        <v>32</v>
+      </c>
+      <c r="D37" s="1" t="s">
+        <v>207</v>
+      </c>
+      <c r="E37" s="15">
+        <v>117</v>
+      </c>
+    </row>
+    <row r="38" spans="2:6" x14ac:dyDescent="0.55000000000000004">
+      <c r="B38" s="15">
+        <v>33</v>
+      </c>
+      <c r="D38" s="1" t="s">
+        <v>208</v>
+      </c>
+    </row>
+    <row r="39" spans="2:6" x14ac:dyDescent="0.55000000000000004">
+      <c r="B39" s="15">
+        <v>34</v>
+      </c>
+      <c r="D39" s="1" t="s">
+        <v>209</v>
+      </c>
+    </row>
+    <row r="40" spans="2:6" x14ac:dyDescent="0.55000000000000004">
+      <c r="B40" s="15">
+        <v>35</v>
+      </c>
+      <c r="D40" s="1" t="s">
+        <v>210</v>
+      </c>
+      <c r="E40" s="15">
+        <v>119</v>
+      </c>
+    </row>
+    <row r="41" spans="2:6" x14ac:dyDescent="0.55000000000000004">
+      <c r="B41" s="15">
+        <v>36</v>
+      </c>
+      <c r="D41" s="1" t="s">
+        <v>211</v>
+      </c>
+      <c r="E41" s="15">
+        <v>120</v>
+      </c>
+    </row>
+    <row r="42" spans="2:6" x14ac:dyDescent="0.55000000000000004">
+      <c r="B42" s="15">
+        <v>37</v>
+      </c>
+      <c r="D42" s="1" t="s">
+        <v>212</v>
+      </c>
+      <c r="E42" s="15">
+        <v>103</v>
+      </c>
+    </row>
+    <row r="43" spans="2:6" x14ac:dyDescent="0.55000000000000004">
+      <c r="B43" s="15">
+        <v>38</v>
+      </c>
+      <c r="D43" s="1" t="s">
+        <v>213</v>
+      </c>
+    </row>
+    <row r="44" spans="2:6" x14ac:dyDescent="0.55000000000000004">
+      <c r="B44" s="15">
+        <v>39</v>
+      </c>
+      <c r="D44" s="1" t="s">
+        <v>214</v>
+      </c>
+    </row>
+    <row r="45" spans="2:6" x14ac:dyDescent="0.55000000000000004">
+      <c r="B45" s="15">
+        <v>40</v>
+      </c>
+      <c r="D45" s="1" t="s">
+        <v>215</v>
+      </c>
+      <c r="E45" s="15">
+        <v>146</v>
+      </c>
+    </row>
+    <row r="46" spans="2:6" x14ac:dyDescent="0.55000000000000004">
+      <c r="B46" s="15">
+        <v>41</v>
+      </c>
+      <c r="D46" s="1" t="s">
+        <v>216</v>
+      </c>
+    </row>
+    <row r="47" spans="2:6" x14ac:dyDescent="0.55000000000000004">
+      <c r="B47" s="15">
+        <v>42</v>
+      </c>
+      <c r="D47" s="1" t="s">
+        <v>217</v>
+      </c>
+      <c r="E47" s="15">
+        <v>148</v>
+      </c>
+    </row>
+    <row r="48" spans="2:6" x14ac:dyDescent="0.55000000000000004">
+      <c r="B48" s="15">
+        <v>43</v>
+      </c>
+      <c r="D48" s="1" t="s">
+        <v>218</v>
+      </c>
+      <c r="F48" s="1" t="s">
+        <v>219</v>
+      </c>
+    </row>
+    <row r="49" spans="2:5" x14ac:dyDescent="0.55000000000000004">
+      <c r="B49" s="15">
+        <v>44</v>
+      </c>
+      <c r="D49" s="1" t="s">
+        <v>221</v>
+      </c>
+    </row>
+    <row r="50" spans="2:5" x14ac:dyDescent="0.55000000000000004">
+      <c r="B50" s="15">
+        <v>45</v>
+      </c>
+      <c r="D50" s="1" t="s">
+        <v>222</v>
+      </c>
+    </row>
+    <row r="51" spans="2:5" x14ac:dyDescent="0.55000000000000004">
+      <c r="B51" s="15">
+        <v>46</v>
+      </c>
+      <c r="D51" s="1" t="s">
+        <v>223</v>
+      </c>
+    </row>
+    <row r="52" spans="2:5" x14ac:dyDescent="0.55000000000000004">
+      <c r="B52" s="15">
+        <v>47</v>
+      </c>
+      <c r="D52" s="1" t="s">
+        <v>224</v>
+      </c>
+    </row>
+    <row r="53" spans="2:5" x14ac:dyDescent="0.55000000000000004">
+      <c r="B53" s="15">
+        <v>48</v>
+      </c>
+      <c r="D53" s="1" t="s">
+        <v>225</v>
+      </c>
+    </row>
+    <row r="54" spans="2:5" x14ac:dyDescent="0.55000000000000004">
+      <c r="B54" s="15">
+        <v>49</v>
+      </c>
+      <c r="D54" s="1" t="s">
+        <v>226</v>
+      </c>
+      <c r="E54" s="15">
+        <v>157</v>
+      </c>
+    </row>
+    <row r="55" spans="2:5" x14ac:dyDescent="0.55000000000000004">
+      <c r="B55" s="15">
+        <v>50</v>
+      </c>
+      <c r="D55" s="1" t="s">
+        <v>227</v>
+      </c>
+      <c r="E55" s="15">
+        <v>163</v>
+      </c>
+    </row>
+    <row r="56" spans="2:5" x14ac:dyDescent="0.55000000000000004">
+      <c r="B56" s="15">
+        <v>51</v>
+      </c>
+      <c r="C56" s="15">
+        <v>1002</v>
+      </c>
+      <c r="D56" s="1" t="s">
+        <v>228</v>
+      </c>
+    </row>
+    <row r="57" spans="2:5" x14ac:dyDescent="0.55000000000000004">
+      <c r="B57" s="15">
+        <v>52</v>
+      </c>
+      <c r="C57" s="15">
+        <v>2</v>
+      </c>
+      <c r="D57" s="1" t="s">
+        <v>191</v>
+      </c>
+    </row>
+  </sheetData>
+  <autoFilter ref="B5:E5" xr:uid="{1D1C1021-2470-4A18-9715-81111F931C52}"/>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <pageSetup orientation="landscape" r:id="rId1"/>
+  <headerFooter>
+    <oddHeader>&amp;L&amp;F&amp;CUNCLASSIFIED&amp;R&amp;A</oddHeader>
+    <oddFooter>&amp;Lprinted: &amp;D&amp;CUNCLASSIFIED&amp;Rpage &amp;P of &amp;N</oddFooter>
+  </headerFooter>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0400-000000000000}">
   <dimension ref="A1:O20"/>
   <sheetFormatPr defaultColWidth="9.15625" defaultRowHeight="14.4" x14ac:dyDescent="0.55000000000000004"/>

</xml_diff>